<commit_message>
adding in rdrp gene build
</commit_message>
<xml_diff>
--- a/config/published_clades.xlsx
+++ b/config/published_clades.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\msomno\Documents\GitHub\HCoV_229E\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2DF9EBE-5DC1-40DC-B39A-8BD476C47632}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EC94C5-A864-4D3C-94DB-36665D09C8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-51705" yWindow="-1905" windowWidth="26010" windowHeight="20985" xr2:uid="{810DED4B-93A4-4169-BBE6-C2803528C88A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{810DED4B-93A4-4169-BBE6-C2803528C88A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$159</definedName>
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">Sheet2!$A$1:$B$1068</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2437" uniqueCount="1819">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2626" uniqueCount="1826">
   <si>
     <t>accession</t>
   </si>
@@ -5502,17 +5502,38 @@
     <t>Ye et al 2016</t>
   </si>
   <si>
-    <t>7a</t>
-  </si>
-  <si>
-    <t>7b</t>
+    <t>PQ616096 </t>
+  </si>
+  <si>
+    <t>Musaeva et al 2024</t>
+  </si>
+  <si>
+    <t>Genotype 6</t>
+  </si>
+  <si>
+    <t>Genotype 7a</t>
+  </si>
+  <si>
+    <t>Genotype 7b</t>
+  </si>
+  <si>
+    <t>Genotype 2</t>
+  </si>
+  <si>
+    <t>Genotype 3</t>
+  </si>
+  <si>
+    <t>Genotype 4</t>
+  </si>
+  <si>
+    <t>Genotype 5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5536,6 +5557,13 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -5554,16 +5582,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{3FF454AD-1D9B-446C-88A9-4A5E6692A50F}"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
@@ -5962,7 +5994,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44BDE173-2FC9-4609-92DD-26580848C26D}">
-  <dimension ref="A1:F113"/>
+  <dimension ref="A1:F159"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
@@ -5999,8 +6031,8 @@
       <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1">
-        <v>6</v>
+      <c r="C2" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -6014,8 +6046,8 @@
       <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="1">
-        <v>6</v>
+      <c r="C3" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>10</v>
@@ -6029,8 +6061,8 @@
       <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1">
-        <v>6</v>
+      <c r="C4" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>10</v>
@@ -6044,8 +6076,8 @@
       <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1">
-        <v>6</v>
+      <c r="C5" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>10</v>
@@ -6060,7 +6092,7 @@
         <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>10</v>
@@ -6075,7 +6107,7 @@
         <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>10</v>
@@ -6090,7 +6122,7 @@
         <v>14</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>10</v>
@@ -6105,7 +6137,7 @@
         <v>12</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>10</v>
@@ -6120,7 +6152,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>10</v>
@@ -6135,7 +6167,7 @@
         <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>10</v>
@@ -6150,7 +6182,7 @@
         <v>17</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>10</v>
@@ -6165,7 +6197,7 @@
         <v>18</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>10</v>
@@ -6180,7 +6212,7 @@
         <v>19</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>10</v>
@@ -6195,7 +6227,7 @@
         <v>20</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>10</v>
@@ -6210,7 +6242,7 @@
         <v>21</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F16" s="1" t="s">
         <v>10</v>
@@ -6225,7 +6257,7 @@
         <v>22</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F17" s="1" t="s">
         <v>10</v>
@@ -6240,7 +6272,7 @@
         <v>23</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>10</v>
@@ -6255,7 +6287,7 @@
         <v>24</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>10</v>
@@ -6270,7 +6302,7 @@
         <v>25</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>10</v>
@@ -6285,7 +6317,7 @@
         <v>26</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>10</v>
@@ -6300,7 +6332,7 @@
         <v>27</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>10</v>
@@ -6315,7 +6347,7 @@
         <v>28</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>10</v>
@@ -6330,7 +6362,7 @@
         <v>29</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>10</v>
@@ -6345,7 +6377,7 @@
         <v>30</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F25" s="1" t="s">
         <v>10</v>
@@ -6360,7 +6392,7 @@
         <v>31</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>10</v>
@@ -6375,7 +6407,7 @@
         <v>39</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F27" s="1" t="s">
         <v>10</v>
@@ -6390,7 +6422,7 @@
         <v>34</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F28" s="1" t="s">
         <v>10</v>
@@ -6405,7 +6437,7 @@
         <v>35</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>10</v>
@@ -6420,7 +6452,7 @@
         <v>36</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F30" s="1" t="s">
         <v>10</v>
@@ -6435,7 +6467,7 @@
         <v>40</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>10</v>
@@ -6450,7 +6482,7 @@
         <v>33</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>10</v>
@@ -6465,7 +6497,7 @@
         <v>41</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F33" s="1" t="s">
         <v>10</v>
@@ -6480,7 +6512,7 @@
         <v>44</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F34" s="1" t="s">
         <v>10</v>
@@ -6495,7 +6527,7 @@
         <v>45</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>10</v>
@@ -6510,7 +6542,7 @@
         <v>43</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>10</v>
@@ -6525,769 +6557,1386 @@
         <v>42</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F37" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C38" s="1">
-        <v>6</v>
+      <c r="A38" s="3" t="s">
+        <v>852</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>852</v>
-      </c>
-      <c r="C39" s="1">
-        <v>6</v>
+      <c r="A39" s="3" t="s">
+        <v>854</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F39" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>854</v>
-      </c>
-      <c r="C40" s="1">
-        <v>6</v>
+      <c r="A40" s="3" t="s">
+        <v>919</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F40" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>919</v>
-      </c>
-      <c r="C41" s="1">
-        <v>6</v>
+      <c r="A41" s="3" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F41" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>1087</v>
-      </c>
-      <c r="C42" s="1">
-        <v>6</v>
+      <c r="A42" s="3" t="s">
+        <v>851</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>851</v>
-      </c>
-      <c r="C43" s="1">
-        <v>6</v>
+      <c r="A43" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>860</v>
-      </c>
-      <c r="C44" s="1">
-        <v>6</v>
+      <c r="A44" s="3" t="s">
+        <v>861</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F44" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>861</v>
-      </c>
-      <c r="C45" s="1">
-        <v>6</v>
+      <c r="A45" s="3" t="s">
+        <v>827</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>1819</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>827</v>
-      </c>
-      <c r="C46" s="1">
-        <v>6</v>
+      <c r="A46" s="3" t="s">
+        <v>849</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>1820</v>
       </c>
       <c r="F46" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>849</v>
+      <c r="A47" s="3" t="s">
+        <v>866</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F47" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
-        <v>866</v>
+      <c r="A48" s="3" t="s">
+        <v>1081</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F48" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
-        <v>1081</v>
+      <c r="A49" s="3" t="s">
+        <v>1083</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F49" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
-        <v>1083</v>
+      <c r="A50" s="3" t="s">
+        <v>1085</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F50" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
-        <v>1085</v>
+      <c r="A51" s="3" t="s">
+        <v>1412</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>1817</v>
+        <v>1820</v>
       </c>
       <c r="F51" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
-        <v>1412</v>
+      <c r="A52" s="3" t="s">
+        <v>864</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F52" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
-        <v>1452</v>
+      <c r="A53" s="3" t="s">
+        <v>856</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F53" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
-        <v>864</v>
+      <c r="A54" s="3" t="s">
+        <v>859</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F54" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
-        <v>856</v>
+      <c r="A55" s="3" t="s">
+        <v>1348</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F55" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
-        <v>859</v>
+      <c r="A56" s="3" t="s">
+        <v>1350</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F56" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
-        <v>1348</v>
+      <c r="A57" s="3" t="s">
+        <v>1352</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F57" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
-        <v>1350</v>
+      <c r="A58" s="3" t="s">
+        <v>1354</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F58" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
-        <v>1352</v>
+      <c r="A59" s="3" t="s">
+        <v>1358</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F59" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
-        <v>1354</v>
+      <c r="A60" s="3" t="s">
+        <v>1360</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F60" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
-        <v>1358</v>
+      <c r="A61" s="3" t="s">
+        <v>1362</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F61" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
-        <v>1360</v>
+      <c r="A62" s="3" t="s">
+        <v>1364</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F62" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>1362</v>
+      <c r="A63" s="3" t="s">
+        <v>1366</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F63" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>1364</v>
+      <c r="A64" s="3" t="s">
+        <v>1386</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F64" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
-        <v>1366</v>
+      <c r="A65" s="3" t="s">
+        <v>1368</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>1386</v>
+      <c r="A66" s="3" t="s">
+        <v>1388</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>1368</v>
+      <c r="A67" s="3" t="s">
+        <v>1390</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>1388</v>
+      <c r="A68" s="3" t="s">
+        <v>1392</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F68" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>1390</v>
+      <c r="A69" s="3" t="s">
+        <v>1394</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F69" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>1392</v>
+      <c r="A70" s="3" t="s">
+        <v>1396</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
-        <v>1394</v>
+      <c r="A71" s="3" t="s">
+        <v>1398</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
-        <v>1396</v>
+      <c r="A72" s="3" t="s">
+        <v>1400</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>1398</v>
+      <c r="A73" s="3" t="s">
+        <v>1402</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>1400</v>
+      <c r="A74" s="3" t="s">
+        <v>1404</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>1402</v>
+      <c r="A75" s="3" t="s">
+        <v>1406</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>1404</v>
+      <c r="A76" s="3" t="s">
+        <v>1416</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F76" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>1406</v>
+      <c r="A77" s="3" t="s">
+        <v>1420</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F77" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
-        <v>1416</v>
+      <c r="A78" s="3" t="s">
+        <v>1422</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F78" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
-        <v>1420</v>
+      <c r="A79" s="3" t="s">
+        <v>1424</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F79" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>1422</v>
+      <c r="A80" s="3" t="s">
+        <v>1426</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F80" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>1424</v>
+      <c r="A81" s="3" t="s">
+        <v>1430</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F81" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
-        <v>1426</v>
+      <c r="A82" s="3" t="s">
+        <v>1344</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F82" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
-        <v>1450</v>
+      <c r="A83" s="1" t="s">
+        <v>925</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="F83" s="1" t="s">
         <v>1816</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
-        <v>1430</v>
+      <c r="A84" s="3" t="s">
+        <v>857</v>
       </c>
       <c r="C84" s="1" t="s">
+        <v>1819</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" s="3" t="s">
+        <v>1414</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" s="3" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" s="3" t="s">
+        <v>1321</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" s="1" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" s="3" t="s">
+        <v>1342</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" s="3" t="s">
+        <v>923</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" s="3" t="s">
+        <v>1428</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" s="1" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" s="3" t="s">
+        <v>1418</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" s="3" t="s">
+        <v>1325</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A96" s="3" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A97" s="3" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A98" s="3" t="s">
+        <v>1327</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A99" s="3" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A100" s="3" t="s">
+        <v>1410</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A101" s="3" t="s">
+        <v>1370</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A102" s="3" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A103" s="3" t="s">
+        <v>1384</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A104" s="3" t="s">
+        <v>1329</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A105" s="3" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A106" s="3" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A107" s="3" t="s">
+        <v>1378</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A108" s="3" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A109" s="3" t="s">
+        <v>1372</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A110" s="3" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A111" s="4" t="s">
+        <v>1450</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>1451</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F111" s="1" t="s">
         <v>1818</v>
       </c>
-      <c r="F84" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
-        <v>1344</v>
-      </c>
-      <c r="C85" s="1" t="s">
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A112" s="4" t="s">
+        <v>1452</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>1453</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F112" s="1" t="s">
         <v>1818</v>
       </c>
-      <c r="F85" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A86" s="1" t="s">
-        <v>925</v>
-      </c>
-      <c r="C86" s="1" t="s">
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A113" s="4" t="s">
+        <v>1454</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>1455</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F113" s="1" t="s">
         <v>1818</v>
       </c>
-      <c r="F86" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
-        <v>857</v>
-      </c>
-      <c r="C87" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
-        <v>865</v>
-      </c>
-      <c r="C88" s="1" t="s">
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A114" s="4" t="s">
+        <v>1456</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>1457</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A115" s="4" t="s">
+        <v>1680</v>
+      </c>
+      <c r="B115" s="4" t="s">
+        <v>1681</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A116" s="4" t="s">
+        <v>1682</v>
+      </c>
+      <c r="B116" s="4" t="s">
+        <v>1683</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A117" s="4" t="s">
+        <v>1684</v>
+      </c>
+      <c r="B117" s="4" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A118" s="4" t="s">
+        <v>1686</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>1687</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A119" s="4" t="s">
+        <v>1688</v>
+      </c>
+      <c r="B119" s="4" t="s">
+        <v>1689</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A120" s="4" t="s">
+        <v>1690</v>
+      </c>
+      <c r="B120" s="4" t="s">
+        <v>1691</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A121" s="4" t="s">
+        <v>1692</v>
+      </c>
+      <c r="B121" s="4" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A122" s="4" t="s">
+        <v>1696</v>
+      </c>
+      <c r="B122" s="4" t="s">
+        <v>1697</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A123" s="4" t="s">
+        <v>1698</v>
+      </c>
+      <c r="B123" s="4" t="s">
+        <v>1699</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A124" s="4" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B124" s="4" t="s">
+        <v>1701</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>1822</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A125" s="4" t="s">
+        <v>1702</v>
+      </c>
+      <c r="B125" s="4" t="s">
+        <v>1703</v>
+      </c>
+      <c r="C125" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A126" s="4" t="s">
+        <v>1704</v>
+      </c>
+      <c r="B126" s="4" t="s">
+        <v>1705</v>
+      </c>
+      <c r="C126" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A127" s="4" t="s">
+        <v>1706</v>
+      </c>
+      <c r="B127" s="4" t="s">
+        <v>1707</v>
+      </c>
+      <c r="C127" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A128" s="4" t="s">
+        <v>1708</v>
+      </c>
+      <c r="B128" s="4" t="s">
+        <v>1709</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A129" s="4" t="s">
+        <v>1710</v>
+      </c>
+      <c r="B129" s="4" t="s">
+        <v>1711</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A130" s="4" t="s">
+        <v>1714</v>
+      </c>
+      <c r="B130" s="4" t="s">
+        <v>1715</v>
+      </c>
+      <c r="C130" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A131" s="4" t="s">
+        <v>1716</v>
+      </c>
+      <c r="B131" s="4" t="s">
+        <v>1717</v>
+      </c>
+      <c r="C131" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A132" s="4" t="s">
+        <v>1718</v>
+      </c>
+      <c r="B132" s="4" t="s">
+        <v>1719</v>
+      </c>
+      <c r="C132" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A133" s="4" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B133" s="4" t="s">
+        <v>1721</v>
+      </c>
+      <c r="C133" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A134" s="4" t="s">
+        <v>1724</v>
+      </c>
+      <c r="B134" s="4" t="s">
+        <v>1725</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A135" s="4" t="s">
         <v>1817</v>
       </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
-        <v>1414</v>
-      </c>
-      <c r="C89" s="1" t="s">
+      <c r="B135" s="4" t="s">
+        <v>1727</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F135" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
-        <v>1408</v>
-      </c>
-      <c r="C90" s="1" t="s">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A136" s="4" t="s">
+        <v>1728</v>
+      </c>
+      <c r="B136" s="4" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F136" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
-        <v>1321</v>
-      </c>
-      <c r="C91" s="1" t="s">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A137" s="4" t="s">
+        <v>1730</v>
+      </c>
+      <c r="B137" s="4" t="s">
+        <v>1731</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F137" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A92" s="1" t="s">
-        <v>1323</v>
-      </c>
-      <c r="C92" s="1" t="s">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A138" s="4" t="s">
+        <v>1734</v>
+      </c>
+      <c r="B138" s="4" t="s">
+        <v>1735</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F138" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
-        <v>1342</v>
-      </c>
-      <c r="C93" s="1" t="s">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A139" s="4" t="s">
+        <v>1736</v>
+      </c>
+      <c r="B139" s="4" t="s">
+        <v>1737</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F139" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
-        <v>923</v>
-      </c>
-      <c r="C94" s="1" t="s">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A140" s="4" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B140" s="4" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F140" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
-        <v>1428</v>
-      </c>
-      <c r="C95" s="1" t="s">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A141" s="4" t="s">
+        <v>1740</v>
+      </c>
+      <c r="B141" s="4" t="s">
+        <v>1741</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F141" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A96" s="1" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C96" s="1" t="s">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A142" s="4" t="s">
+        <v>1742</v>
+      </c>
+      <c r="B142" s="4" t="s">
+        <v>1743</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F142" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
-        <v>1418</v>
-      </c>
-      <c r="C97" s="1" t="s">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A143" s="4" t="s">
+        <v>1744</v>
+      </c>
+      <c r="B143" s="4" t="s">
+        <v>1745</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F143" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
-        <v>1325</v>
-      </c>
-      <c r="C98" s="1" t="s">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A144" s="4" t="s">
+        <v>1746</v>
+      </c>
+      <c r="B144" s="4" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F144" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
-        <v>1317</v>
-      </c>
-      <c r="C99" s="1" t="s">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A145" s="4" t="s">
+        <v>1748</v>
+      </c>
+      <c r="B145" s="4" t="s">
+        <v>1749</v>
+      </c>
+      <c r="C145" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F145" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
-        <v>1319</v>
-      </c>
-      <c r="C100" s="1" t="s">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A146" s="4" t="s">
+        <v>1750</v>
+      </c>
+      <c r="B146" s="4" t="s">
+        <v>1751</v>
+      </c>
+      <c r="C146" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F146" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
-        <v>1327</v>
-      </c>
-      <c r="C101" s="1" t="s">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A147" s="4" t="s">
+        <v>1752</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>1753</v>
+      </c>
+      <c r="C147" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F147" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
-        <v>1315</v>
-      </c>
-      <c r="C102" s="1" t="s">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A148" s="4" t="s">
+        <v>1754</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>1755</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F148" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
-        <v>1410</v>
-      </c>
-      <c r="C103" s="1" t="s">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A149" s="4" t="s">
+        <v>1756</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>1757</v>
+      </c>
+      <c r="C149" s="4" t="s">
+        <v>1821</v>
+      </c>
+      <c r="F149" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
-        <v>1370</v>
-      </c>
-      <c r="C104" s="1" t="s">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A150" s="1" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>1822</v>
+      </c>
+      <c r="F150" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C105" s="1" t="s">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A151" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>1823</v>
+      </c>
+      <c r="F151" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A106" t="s">
-        <v>1384</v>
-      </c>
-      <c r="C106" s="1" t="s">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A152" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>1823</v>
+      </c>
+      <c r="F152" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
-        <v>1329</v>
-      </c>
-      <c r="C107" s="1" t="s">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A153" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>1823</v>
+      </c>
+      <c r="F153" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A108" t="s">
-        <v>1346</v>
-      </c>
-      <c r="C108" s="1" t="s">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A154" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>1823</v>
+      </c>
+      <c r="F154" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A109" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C109" s="1" t="s">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A155" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>1823</v>
+      </c>
+      <c r="F155" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A110" t="s">
-        <v>1378</v>
-      </c>
-      <c r="C110" s="1" t="s">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A156" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C156" s="1" t="s">
+        <v>1824</v>
+      </c>
+      <c r="F156" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A111" t="s">
-        <v>1382</v>
-      </c>
-      <c r="C111" s="1" t="s">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A157" s="1" t="s">
+        <v>862</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>1824</v>
+      </c>
+      <c r="F157" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A112" t="s">
-        <v>1372</v>
-      </c>
-      <c r="C112" s="1" t="s">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A158" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>1825</v>
+      </c>
+      <c r="F158" s="1" t="s">
         <v>1818</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A113" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>1818</v>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A159" s="1" t="s">
+        <v>1079</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:C113" xr:uid="{44BDE173-2FC9-4609-92DD-26580848C26D}"/>
+  <autoFilter ref="C1:C159" xr:uid="{44BDE173-2FC9-4609-92DD-26580848C26D}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>

<commit_message>
updated refine and config files
</commit_message>
<xml_diff>
--- a/config/published_clades.xlsx
+++ b/config/published_clades.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\msomno\Documents\GitHub\HCoV_229E\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3EC94C5-A864-4D3C-94DB-36665D09C8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD6962D-A70E-4EAE-B2E2-0F4020484681}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{810DED4B-93A4-4169-BBE6-C2803528C88A}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$159</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$149</definedName>
     <definedName name="ExternalData_1" localSheetId="1" hidden="1">Sheet2!$A$1:$B$1068</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2626" uniqueCount="1826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2604" uniqueCount="1832">
   <si>
     <t>accession</t>
   </si>
@@ -5499,9 +5499,6 @@
     <t>LRI 281</t>
   </si>
   <si>
-    <t>Ye et al 2016</t>
-  </si>
-  <si>
     <t>PQ616096 </t>
   </si>
   <si>
@@ -5527,6 +5524,27 @@
   </si>
   <si>
     <t>Genotype 5</t>
+  </si>
+  <si>
+    <t>KY36991</t>
+  </si>
+  <si>
+    <t>KY36990</t>
+  </si>
+  <si>
+    <t>KY96735</t>
+  </si>
+  <si>
+    <t>KY98358</t>
+  </si>
+  <si>
+    <t>ON55409</t>
+  </si>
+  <si>
+    <t>OK07307</t>
+  </si>
+  <si>
+    <t>ON55411</t>
   </si>
 </sst>
 </file>
@@ -5586,18 +5604,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{3FF454AD-1D9B-446C-88A9-4A5E6692A50F}"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -5670,8 +5697,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{07817CD8-F663-476C-9983-781063751623}" name="metadata" displayName="metadata" ref="A1:B1068" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:B1068" xr:uid="{07817CD8-F663-476C-9983-781063751623}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{6A4C8813-EFEE-485D-ADDC-25B402AE7B2E}" uniqueName="1" name="accession" queryTableFieldId="1" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{1FD82F6C-26C2-4B34-BD48-D3FB581DDA8E}" uniqueName="5" name="strain" queryTableFieldId="5" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{6A4C8813-EFEE-485D-ADDC-25B402AE7B2E}" uniqueName="1" name="accession" queryTableFieldId="1" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{1FD82F6C-26C2-4B34-BD48-D3FB581DDA8E}" uniqueName="5" name="strain" queryTableFieldId="5" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5994,7 +6021,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44BDE173-2FC9-4609-92DD-26580848C26D}">
-  <dimension ref="A1:F159"/>
+  <dimension ref="A1:F149"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
@@ -6032,7 +6059,7 @@
         <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>10</v>
@@ -6047,7 +6074,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>10</v>
@@ -6062,7 +6089,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>10</v>
@@ -6077,7 +6104,7 @@
         <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>1819</v>
+        <v>1818</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>10</v>
@@ -6092,7 +6119,7 @@
         <v>11</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>10</v>
@@ -6107,7 +6134,7 @@
         <v>13</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>10</v>
@@ -6122,7 +6149,7 @@
         <v>14</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>10</v>
@@ -6137,7 +6164,7 @@
         <v>12</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>10</v>
@@ -6152,7 +6179,7 @@
         <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>10</v>
@@ -6167,112 +6194,70 @@
         <v>16</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="str">
-        <f>INDEX(Sheet2!A:A, MATCH(B12, Sheet2!B:B, 0))</f>
-        <v>PQ466800</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>17</v>
+      <c r="A12" s="1" t="s">
+        <v>1826</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>1820</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>10</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="str">
-        <f>INDEX(Sheet2!A:A, MATCH(B13, Sheet2!B:B, 0))</f>
-        <v>PQ466805</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>18</v>
+      <c r="A13" t="s">
+        <v>1827</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>1820</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>10</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="str">
-        <f>INDEX(Sheet2!A:A, MATCH(B14, Sheet2!B:B, 0))</f>
-        <v>PQ466836</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>19</v>
+      <c r="A14" t="s">
+        <v>1828</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>1820</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>10</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" s="1" t="str">
-        <f>INDEX(Sheet2!A:A, MATCH(B15, Sheet2!B:B, 0))</f>
-        <v>PQ466838</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>20</v>
+      <c r="A15" t="s">
+        <v>1081</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>1820</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>10</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="str">
-        <f>INDEX(Sheet2!A:A, MATCH(B16, Sheet2!B:B, 0))</f>
-        <v>PQ466841</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>21</v>
+      <c r="A16" t="s">
+        <v>1085</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>1820</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>10</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="str">
-        <f>INDEX(Sheet2!A:A, MATCH(B17, Sheet2!B:B, 0))</f>
-        <v>PQ466833</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>22</v>
+      <c r="A17" t="s">
+        <v>1083</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>1820</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>10</v>
+        <v>1819</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B18, Sheet2!B:B, 0))</f>
-        <v>PQ466825</v>
+        <v>PQ466800</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>10</v>
@@ -6281,13 +6266,13 @@
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B19, Sheet2!B:B, 0))</f>
-        <v>PQ466793</v>
+        <v>PQ466805</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>10</v>
@@ -6296,13 +6281,13 @@
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B20, Sheet2!B:B, 0))</f>
-        <v>PQ466813</v>
+        <v>PQ466836</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>10</v>
@@ -6311,13 +6296,13 @@
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B21, Sheet2!B:B, 0))</f>
-        <v>PQ466814</v>
+        <v>PQ466838</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>10</v>
@@ -6326,13 +6311,13 @@
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B22, Sheet2!B:B, 0))</f>
-        <v>PQ466824</v>
+        <v>PQ466841</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>10</v>
@@ -6341,13 +6326,13 @@
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B23, Sheet2!B:B, 0))</f>
-        <v>PQ466827</v>
+        <v>PQ466833</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F23" s="1" t="s">
         <v>10</v>
@@ -6356,13 +6341,13 @@
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B24, Sheet2!B:B, 0))</f>
-        <v>PQ466804</v>
+        <v>PQ466825</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>10</v>
@@ -6371,10 +6356,10 @@
     <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B25, Sheet2!B:B, 0))</f>
-        <v>PQ466810</v>
+        <v>PQ466793</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>1820</v>
@@ -6386,10 +6371,10 @@
     <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B26, Sheet2!B:B, 0))</f>
-        <v>PQ466839</v>
+        <v>PQ466813</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>1820</v>
@@ -6401,10 +6386,10 @@
     <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B27, Sheet2!B:B, 0))</f>
-        <v>PQ466851</v>
+        <v>PQ466814</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>1820</v>
@@ -6416,10 +6401,10 @@
     <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B28, Sheet2!B:B, 0))</f>
-        <v>PQ466848</v>
+        <v>PQ466824</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>1820</v>
@@ -6431,13 +6416,13 @@
     <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B29, Sheet2!B:B, 0))</f>
-        <v>PQ466849</v>
+        <v>PQ466827</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>1820</v>
+        <v>1819</v>
       </c>
       <c r="F29" s="1" t="s">
         <v>10</v>
@@ -6446,10 +6431,10 @@
     <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B30, Sheet2!B:B, 0))</f>
-        <v>PQ466847</v>
+        <v>PQ466804</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>1820</v>
@@ -6461,10 +6446,10 @@
     <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B31, Sheet2!B:B, 0))</f>
-        <v>PQ466854</v>
+        <v>PQ466810</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>1820</v>
@@ -6476,10 +6461,10 @@
     <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B32, Sheet2!B:B, 0))</f>
-        <v>PQ466842</v>
+        <v>PQ466839</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>1820</v>
@@ -6491,10 +6476,10 @@
     <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B33, Sheet2!B:B, 0))</f>
-        <v>PQ466852</v>
+        <v>PQ466851</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>1820</v>
@@ -6506,10 +6491,10 @@
     <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B34, Sheet2!B:B, 0))</f>
-        <v>PQ466855</v>
+        <v>PQ466848</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>1820</v>
@@ -6521,10 +6506,10 @@
     <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B35, Sheet2!B:B, 0))</f>
-        <v>PQ466856</v>
+        <v>PQ466849</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>1820</v>
@@ -6536,10 +6521,10 @@
     <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B36, Sheet2!B:B, 0))</f>
-        <v>PQ466857</v>
+        <v>PQ466847</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>1820</v>
@@ -6551,10 +6536,10 @@
     <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="str">
         <f>INDEX(Sheet2!A:A, MATCH(B37, Sheet2!B:B, 0))</f>
-        <v>PQ466853</v>
+        <v>PQ466854</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>1820</v>
@@ -6564,1382 +6549,1341 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A38" s="3" t="s">
-        <v>852</v>
+      <c r="A38" s="1" t="str">
+        <f>INDEX(Sheet2!A:A, MATCH(B38, Sheet2!B:B, 0))</f>
+        <v>PQ466842</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>33</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A39" s="3" t="s">
-        <v>854</v>
+      <c r="A39" s="1" t="str">
+        <f>INDEX(Sheet2!A:A, MATCH(B39, Sheet2!B:B, 0))</f>
+        <v>PQ466852</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A40" s="3" t="s">
-        <v>919</v>
+      <c r="A40" s="1" t="str">
+        <f>INDEX(Sheet2!A:A, MATCH(B40, Sheet2!B:B, 0))</f>
+        <v>PQ466855</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A41" s="3" t="s">
-        <v>1087</v>
+      <c r="A41" s="1" t="str">
+        <f>INDEX(Sheet2!A:A, MATCH(B41, Sheet2!B:B, 0))</f>
+        <v>PQ466856</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A42" s="3" t="s">
-        <v>851</v>
+      <c r="A42" s="1" t="str">
+        <f>INDEX(Sheet2!A:A, MATCH(B42, Sheet2!B:B, 0))</f>
+        <v>PQ466857</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A43" s="3" t="s">
-        <v>860</v>
+      <c r="A43" s="1" t="str">
+        <f>INDEX(Sheet2!A:A, MATCH(B43, Sheet2!B:B, 0))</f>
+        <v>PQ466853</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>42</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A44" s="3" t="s">
-        <v>861</v>
+      <c r="A44" t="s">
+        <v>1414</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A45" s="3" t="s">
-        <v>827</v>
+      <c r="A45" t="s">
+        <v>1412</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>1819</v>
+        <v>1820</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A46" s="3" t="s">
-        <v>849</v>
+      <c r="A46" t="s">
+        <v>864</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A47" s="3" t="s">
-        <v>866</v>
+      <c r="A47" t="s">
+        <v>856</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A48" s="3" t="s">
-        <v>1081</v>
+      <c r="A48" t="s">
+        <v>859</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A49" s="3" t="s">
-        <v>1083</v>
+      <c r="A49" t="s">
+        <v>1348</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A50" s="3" t="s">
-        <v>1085</v>
+      <c r="A50" t="s">
+        <v>1354</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A51" s="3" t="s">
-        <v>1412</v>
+      <c r="A51" t="s">
+        <v>1352</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A52" s="3" t="s">
-        <v>864</v>
+      <c r="A52" t="s">
+        <v>1390</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A53" s="3" t="s">
-        <v>856</v>
+      <c r="A53" t="s">
+        <v>1396</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A54" s="3" t="s">
-        <v>859</v>
+      <c r="A54" t="s">
+        <v>1829</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A55" s="3" t="s">
-        <v>1348</v>
+      <c r="A55" t="s">
+        <v>1362</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A56" s="3" t="s">
-        <v>1350</v>
+      <c r="A56" s="1" t="s">
+        <v>1321</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A57" s="3" t="s">
-        <v>1352</v>
+      <c r="A57" t="s">
+        <v>1323</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A58" s="3" t="s">
-        <v>1354</v>
+      <c r="A58" t="s">
+        <v>1342</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A59" s="3" t="s">
-        <v>1358</v>
+      <c r="A59" t="s">
+        <v>1392</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A60" s="3" t="s">
-        <v>1360</v>
+      <c r="A60" t="s">
+        <v>923</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A61" s="3" t="s">
-        <v>1362</v>
+      <c r="A61" t="s">
+        <v>1111</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A62" s="3" t="s">
-        <v>1364</v>
+      <c r="A62" s="1" t="s">
+        <v>1428</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A63" s="3" t="s">
-        <v>1366</v>
+      <c r="A63" t="s">
+        <v>1422</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A64" s="3" t="s">
-        <v>1386</v>
+      <c r="A64" t="s">
+        <v>1426</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A65" s="3" t="s">
-        <v>1368</v>
+      <c r="A65" t="s">
+        <v>1398</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A66" s="3" t="s">
-        <v>1388</v>
+      <c r="A66" t="s">
+        <v>1404</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A67" s="3" t="s">
-        <v>1390</v>
+      <c r="A67" t="s">
+        <v>1830</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A68" s="3" t="s">
-        <v>1392</v>
+      <c r="A68" t="s">
+        <v>1400</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A69" s="3" t="s">
-        <v>1394</v>
+      <c r="A69" t="s">
+        <v>1327</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A70" s="3" t="s">
-        <v>1396</v>
+      <c r="A70" t="s">
+        <v>925</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A71" s="3" t="s">
-        <v>1398</v>
+      <c r="A71" t="s">
+        <v>1386</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A72" s="3" t="s">
-        <v>1400</v>
+      <c r="A72" t="s">
+        <v>1388</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A73" s="3" t="s">
-        <v>1402</v>
+      <c r="A73" t="s">
+        <v>1410</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A74" s="3" t="s">
-        <v>1404</v>
+      <c r="A74" t="s">
+        <v>1380</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A75" s="3" t="s">
-        <v>1406</v>
+      <c r="A75" t="s">
+        <v>1329</v>
       </c>
       <c r="C75" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A76" s="3" t="s">
-        <v>1416</v>
+      <c r="A76" t="s">
+        <v>1831</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A77" s="3" t="s">
-        <v>1420</v>
+      <c r="A77" t="s">
+        <v>1376</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>1820</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>1816</v>
+        <v>10</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A78" s="3" t="s">
-        <v>1422</v>
+      <c r="A78" t="s">
+        <v>1079</v>
       </c>
       <c r="C78" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>852</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>854</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>919</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>851</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>860</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>861</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>1825</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>827</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>1818</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>857</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
+        <v>865</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>1819</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>1820</v>
       </c>
-      <c r="F78" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A79" s="3" t="s">
-        <v>1424</v>
-      </c>
-      <c r="C79" s="1" t="s">
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>1418</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>1820</v>
       </c>
-      <c r="F79" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A80" s="3" t="s">
-        <v>1426</v>
-      </c>
-      <c r="C80" s="1" t="s">
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>1325</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>1820</v>
       </c>
-      <c r="F80" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A81" s="3" t="s">
-        <v>1430</v>
-      </c>
-      <c r="C81" s="1" t="s">
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>1820</v>
       </c>
-      <c r="F81" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A82" s="3" t="s">
-        <v>1344</v>
-      </c>
-      <c r="C82" s="1" t="s">
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>1319</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>1820</v>
       </c>
-      <c r="F82" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A83" s="1" t="s">
-        <v>925</v>
-      </c>
-      <c r="C83" s="1" t="s">
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>1315</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>1820</v>
       </c>
-      <c r="F83" s="1" t="s">
-        <v>1816</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A84" s="3" t="s">
-        <v>857</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>1819</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A85" s="3" t="s">
-        <v>865</v>
-      </c>
-      <c r="C85" s="1" t="s">
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>1370</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>1820</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A86" s="3" t="s">
-        <v>1414</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A87" s="3" t="s">
-        <v>1408</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A88" s="3" t="s">
-        <v>1321</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A89" s="1" t="s">
-        <v>1323</v>
-      </c>
-      <c r="C89" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A90" s="3" t="s">
-        <v>1342</v>
-      </c>
-      <c r="C90" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A91" s="3" t="s">
-        <v>923</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A92" s="3" t="s">
-        <v>1428</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A93" s="1" t="s">
-        <v>1111</v>
-      </c>
-      <c r="C93" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A94" s="3" t="s">
-        <v>1418</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A95" s="3" t="s">
-        <v>1325</v>
-      </c>
-      <c r="C95" s="1" t="s">
-        <v>1821</v>
-      </c>
-    </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A96" s="3" t="s">
-        <v>1317</v>
+      <c r="A96" t="s">
+        <v>1384</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A97" s="3" t="s">
-        <v>1319</v>
+      <c r="A97" t="s">
+        <v>1346</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A98" s="3" t="s">
-        <v>1327</v>
+      <c r="A98" t="s">
+        <v>1374</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A99" s="3" t="s">
-        <v>1315</v>
+      <c r="A99" t="s">
+        <v>1378</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A100" s="3" t="s">
-        <v>1410</v>
+      <c r="A100" t="s">
+        <v>1382</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A101" s="3" t="s">
-        <v>1370</v>
+      <c r="A101" t="s">
+        <v>1372</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" s="3" t="s">
-        <v>1380</v>
+        <v>1450</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>1451</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" s="3" t="s">
-        <v>1384</v>
+        <v>1452</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>1453</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" s="3" t="s">
-        <v>1329</v>
+        <v>1454</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>1455</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" s="3" t="s">
-        <v>1346</v>
+        <v>1456</v>
+      </c>
+      <c r="B105" s="3" t="s">
+        <v>1457</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" s="3" t="s">
-        <v>1374</v>
+        <v>1680</v>
+      </c>
+      <c r="B106" s="3" t="s">
+        <v>1681</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" s="3" t="s">
-        <v>1378</v>
+        <v>1682</v>
+      </c>
+      <c r="B107" s="3" t="s">
+        <v>1683</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" s="3" t="s">
-        <v>1382</v>
+        <v>1684</v>
+      </c>
+      <c r="B108" s="3" t="s">
+        <v>1685</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" s="3" t="s">
-        <v>1372</v>
+        <v>1686</v>
+      </c>
+      <c r="B109" s="3" t="s">
+        <v>1687</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>1821</v>
+        <v>1820</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>1817</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" s="3" t="s">
-        <v>1376</v>
+        <v>1688</v>
+      </c>
+      <c r="B110" s="3" t="s">
+        <v>1689</v>
       </c>
       <c r="C110" s="1" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A111" s="3" t="s">
+        <v>1690</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>1691</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A112" s="3" t="s">
+        <v>1692</v>
+      </c>
+      <c r="B112" s="3" t="s">
+        <v>1693</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A113" s="3" t="s">
+        <v>1696</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>1697</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A114" s="3" t="s">
+        <v>1698</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>1699</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A115" s="3" t="s">
+        <v>1700</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>1701</v>
+      </c>
+      <c r="C115" s="3" t="s">
         <v>1821</v>
       </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A111" s="4" t="s">
-        <v>1450</v>
-      </c>
-      <c r="B111" s="4" t="s">
-        <v>1451</v>
-      </c>
-      <c r="C111" s="1" t="s">
+      <c r="F115" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A116" s="3" t="s">
+        <v>1702</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>1703</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A117" s="3" t="s">
+        <v>1704</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>1705</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A118" s="3" t="s">
+        <v>1706</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>1707</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A119" s="3" t="s">
+        <v>1708</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>1709</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A120" s="3" t="s">
+        <v>1710</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>1711</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A121" s="3" t="s">
+        <v>1714</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>1715</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A122" s="3" t="s">
+        <v>1716</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>1717</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A123" s="3" t="s">
+        <v>1718</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>1719</v>
+      </c>
+      <c r="C123" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A124" s="3" t="s">
+        <v>1720</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>1721</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A125" s="3" t="s">
+        <v>1724</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>1725</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A126" s="3" t="s">
+        <v>1816</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>1727</v>
+      </c>
+      <c r="C126" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A127" s="3" t="s">
+        <v>1728</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C127" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A128" s="3" t="s">
+        <v>1730</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>1731</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A129" s="3" t="s">
+        <v>1734</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>1735</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A130" s="3" t="s">
+        <v>1736</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>1737</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A131" s="3" t="s">
+        <v>1738</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>1739</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A132" s="3" t="s">
+        <v>1740</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>1741</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A133" s="3" t="s">
+        <v>1742</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>1743</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A134" s="3" t="s">
+        <v>1744</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>1745</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A135" s="3" t="s">
+        <v>1746</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>1747</v>
+      </c>
+      <c r="C135" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A136" s="3" t="s">
+        <v>1748</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>1749</v>
+      </c>
+      <c r="C136" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A137" s="3" t="s">
+        <v>1750</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>1751</v>
+      </c>
+      <c r="C137" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A138" s="3" t="s">
+        <v>1752</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>1753</v>
+      </c>
+      <c r="C138" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A139" s="3" t="s">
+        <v>1754</v>
+      </c>
+      <c r="B139" s="3" t="s">
+        <v>1755</v>
+      </c>
+      <c r="C139" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A140" s="3" t="s">
+        <v>1756</v>
+      </c>
+      <c r="B140" s="3" t="s">
+        <v>1757</v>
+      </c>
+      <c r="C140" s="3" t="s">
+        <v>1820</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A141" s="1" t="s">
+        <v>1331</v>
+      </c>
+      <c r="C141" s="3" t="s">
         <v>1821</v>
       </c>
-      <c r="F111" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A112" s="4" t="s">
-        <v>1452</v>
-      </c>
-      <c r="B112" s="4" t="s">
-        <v>1453</v>
-      </c>
-      <c r="C112" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F112" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A113" s="4" t="s">
-        <v>1454</v>
-      </c>
-      <c r="B113" s="4" t="s">
-        <v>1455</v>
-      </c>
-      <c r="C113" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F113" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A114" s="4" t="s">
-        <v>1456</v>
-      </c>
-      <c r="B114" s="4" t="s">
-        <v>1457</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A115" s="4" t="s">
-        <v>1680</v>
-      </c>
-      <c r="B115" s="4" t="s">
-        <v>1681</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A116" s="4" t="s">
-        <v>1682</v>
-      </c>
-      <c r="B116" s="4" t="s">
-        <v>1683</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F116" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A117" s="4" t="s">
-        <v>1684</v>
-      </c>
-      <c r="B117" s="4" t="s">
-        <v>1685</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F117" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A118" s="4" t="s">
-        <v>1686</v>
-      </c>
-      <c r="B118" s="4" t="s">
-        <v>1687</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F118" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A119" s="4" t="s">
-        <v>1688</v>
-      </c>
-      <c r="B119" s="4" t="s">
-        <v>1689</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F119" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A120" s="4" t="s">
-        <v>1690</v>
-      </c>
-      <c r="B120" s="4" t="s">
-        <v>1691</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F120" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A121" s="4" t="s">
-        <v>1692</v>
-      </c>
-      <c r="B121" s="4" t="s">
-        <v>1693</v>
-      </c>
-      <c r="C121" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F121" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A122" s="4" t="s">
-        <v>1696</v>
-      </c>
-      <c r="B122" s="4" t="s">
-        <v>1697</v>
-      </c>
-      <c r="C122" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F122" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A123" s="4" t="s">
-        <v>1698</v>
-      </c>
-      <c r="B123" s="4" t="s">
-        <v>1699</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F123" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A124" s="4" t="s">
-        <v>1700</v>
-      </c>
-      <c r="B124" s="4" t="s">
-        <v>1701</v>
-      </c>
-      <c r="C124" s="4" t="s">
+      <c r="F141" s="1" t="s">
+        <v>1817</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A142" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C142" s="1" t="s">
         <v>1822</v>
       </c>
-      <c r="F124" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A125" s="4" t="s">
-        <v>1702</v>
-      </c>
-      <c r="B125" s="4" t="s">
-        <v>1703</v>
-      </c>
-      <c r="C125" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F125" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A126" s="4" t="s">
-        <v>1704</v>
-      </c>
-      <c r="B126" s="4" t="s">
-        <v>1705</v>
-      </c>
-      <c r="C126" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F126" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A127" s="4" t="s">
-        <v>1706</v>
-      </c>
-      <c r="B127" s="4" t="s">
-        <v>1707</v>
-      </c>
-      <c r="C127" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F127" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A128" s="4" t="s">
-        <v>1708</v>
-      </c>
-      <c r="B128" s="4" t="s">
-        <v>1709</v>
-      </c>
-      <c r="C128" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F128" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A129" s="4" t="s">
-        <v>1710</v>
-      </c>
-      <c r="B129" s="4" t="s">
-        <v>1711</v>
-      </c>
-      <c r="C129" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F129" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A130" s="4" t="s">
-        <v>1714</v>
-      </c>
-      <c r="B130" s="4" t="s">
-        <v>1715</v>
-      </c>
-      <c r="C130" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F130" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A131" s="4" t="s">
-        <v>1716</v>
-      </c>
-      <c r="B131" s="4" t="s">
-        <v>1717</v>
-      </c>
-      <c r="C131" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F131" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A132" s="4" t="s">
-        <v>1718</v>
-      </c>
-      <c r="B132" s="4" t="s">
-        <v>1719</v>
-      </c>
-      <c r="C132" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F132" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A133" s="4" t="s">
-        <v>1720</v>
-      </c>
-      <c r="B133" s="4" t="s">
-        <v>1721</v>
-      </c>
-      <c r="C133" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F133" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A134" s="4" t="s">
-        <v>1724</v>
-      </c>
-      <c r="B134" s="4" t="s">
-        <v>1725</v>
-      </c>
-      <c r="C134" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F134" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A135" s="4" t="s">
+      <c r="F142" s="1" t="s">
         <v>1817</v>
       </c>
-      <c r="B135" s="4" t="s">
-        <v>1727</v>
-      </c>
-      <c r="C135" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F135" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A136" s="4" t="s">
-        <v>1728</v>
-      </c>
-      <c r="B136" s="4" t="s">
-        <v>1729</v>
-      </c>
-      <c r="C136" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F136" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A137" s="4" t="s">
-        <v>1730</v>
-      </c>
-      <c r="B137" s="4" t="s">
-        <v>1731</v>
-      </c>
-      <c r="C137" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F137" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A138" s="4" t="s">
-        <v>1734</v>
-      </c>
-      <c r="B138" s="4" t="s">
-        <v>1735</v>
-      </c>
-      <c r="C138" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F138" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A139" s="4" t="s">
-        <v>1736</v>
-      </c>
-      <c r="B139" s="4" t="s">
-        <v>1737</v>
-      </c>
-      <c r="C139" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F139" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A140" s="4" t="s">
-        <v>1738</v>
-      </c>
-      <c r="B140" s="4" t="s">
-        <v>1739</v>
-      </c>
-      <c r="C140" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F140" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A141" s="4" t="s">
-        <v>1740</v>
-      </c>
-      <c r="B141" s="4" t="s">
-        <v>1741</v>
-      </c>
-      <c r="C141" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F141" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A142" s="4" t="s">
-        <v>1742</v>
-      </c>
-      <c r="B142" s="4" t="s">
-        <v>1743</v>
-      </c>
-      <c r="C142" s="4" t="s">
-        <v>1821</v>
-      </c>
-      <c r="F142" s="1" t="s">
-        <v>1818</v>
-      </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A143" s="4" t="s">
-        <v>1744</v>
-      </c>
-      <c r="B143" s="4" t="s">
-        <v>1745</v>
-      </c>
-      <c r="C143" s="4" t="s">
-        <v>1821</v>
+      <c r="A143" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>1822</v>
       </c>
       <c r="F143" s="1" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A144" s="4" t="s">
-        <v>1746</v>
-      </c>
-      <c r="B144" s="4" t="s">
-        <v>1747</v>
-      </c>
-      <c r="C144" s="4" t="s">
-        <v>1821</v>
+      <c r="A144" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>1822</v>
       </c>
       <c r="F144" s="1" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A145" s="4" t="s">
-        <v>1748</v>
-      </c>
-      <c r="B145" s="4" t="s">
-        <v>1749</v>
-      </c>
-      <c r="C145" s="4" t="s">
-        <v>1821</v>
+      <c r="A145" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>1822</v>
       </c>
       <c r="F145" s="1" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A146" s="4" t="s">
-        <v>1750</v>
-      </c>
-      <c r="B146" s="4" t="s">
-        <v>1751</v>
-      </c>
-      <c r="C146" s="4" t="s">
-        <v>1821</v>
+      <c r="A146" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>1822</v>
       </c>
       <c r="F146" s="1" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A147" s="4" t="s">
-        <v>1752</v>
-      </c>
-      <c r="B147" s="4" t="s">
-        <v>1753</v>
-      </c>
-      <c r="C147" s="4" t="s">
-        <v>1821</v>
+      <c r="A147" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>1823</v>
       </c>
       <c r="F147" s="1" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A148" s="4" t="s">
-        <v>1754</v>
-      </c>
-      <c r="B148" s="4" t="s">
-        <v>1755</v>
-      </c>
-      <c r="C148" s="4" t="s">
-        <v>1821</v>
+      <c r="A148" s="1" t="s">
+        <v>862</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>1823</v>
       </c>
       <c r="F148" s="1" t="s">
-        <v>1818</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A149" s="4" t="s">
-        <v>1756</v>
-      </c>
-      <c r="B149" s="4" t="s">
-        <v>1757</v>
-      </c>
-      <c r="C149" s="4" t="s">
-        <v>1821</v>
+      <c r="A149" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>1824</v>
       </c>
       <c r="F149" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A150" s="1" t="s">
-        <v>1331</v>
-      </c>
-      <c r="C150" s="4" t="s">
-        <v>1822</v>
-      </c>
-      <c r="F150" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A151" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="C151" s="1" t="s">
-        <v>1823</v>
-      </c>
-      <c r="F151" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A152" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="C152" s="1" t="s">
-        <v>1823</v>
-      </c>
-      <c r="F152" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A153" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="C153" s="1" t="s">
-        <v>1823</v>
-      </c>
-      <c r="F153" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A154" s="1" t="s">
-        <v>352</v>
-      </c>
-      <c r="C154" s="1" t="s">
-        <v>1823</v>
-      </c>
-      <c r="F154" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A155" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="C155" s="1" t="s">
-        <v>1823</v>
-      </c>
-      <c r="F155" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A156" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="C156" s="1" t="s">
-        <v>1824</v>
-      </c>
-      <c r="F156" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A157" s="1" t="s">
-        <v>862</v>
-      </c>
-      <c r="C157" s="1" t="s">
-        <v>1824</v>
-      </c>
-      <c r="F157" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A158" s="1" t="s">
-        <v>317</v>
-      </c>
-      <c r="C158" s="1" t="s">
-        <v>1825</v>
-      </c>
-      <c r="F158" s="1" t="s">
-        <v>1818</v>
-      </c>
-    </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A159" s="1" t="s">
-        <v>1079</v>
+        <v>1817</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:C159" xr:uid="{44BDE173-2FC9-4609-92DD-26580848C26D}"/>
+  <autoFilter ref="C1:C149" xr:uid="{44BDE173-2FC9-4609-92DD-26580848C26D}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A87:A1048576 A56 A1:A12 A18:A43 A62">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>